<commit_message>
walk through WGCNA module building, defining every term on the way
</commit_message>
<xml_diff>
--- a/01_Processing/06_Module_Building/c_data/module_building.xlsx
+++ b/01_Processing/06_Module_Building/c_data/module_building.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6216" uniqueCount="4114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6225" uniqueCount="4120">
   <si>
     <t>sheet</t>
   </si>
@@ -12071,6 +12071,12 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
     <t>knitr</t>
   </si>
   <si>
@@ -12335,6 +12341,12 @@
     <t>0.5.0</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -12363,6 +12375,12 @@
   </si>
   <si>
     <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -42077,7 +42095,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -42613,7 +42631,7 @@
         <v>4022</v>
       </c>
       <c r="B49" t="s">
-        <v>3972</v>
+        <v>4023</v>
       </c>
       <c r="C49" t="s">
         <v>3929</v>
@@ -42621,10 +42639,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>4023</v>
+        <v>4024</v>
       </c>
       <c r="B50" t="s">
-        <v>4024</v>
+        <v>3972</v>
       </c>
       <c r="C50" t="s">
         <v>3929</v>
@@ -42770,7 +42788,7 @@
         <v>4050</v>
       </c>
       <c r="C63" t="s">
-        <v>3934</v>
+        <v>3929</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -42781,7 +42799,7 @@
         <v>4052</v>
       </c>
       <c r="C64" t="s">
-        <v>3929</v>
+        <v>3934</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -42888,10 +42906,10 @@
         <v>4071</v>
       </c>
       <c r="B74" t="s">
-        <v>3976</v>
+        <v>4072</v>
       </c>
       <c r="C74" t="s">
-        <v>4072</v>
+        <v>3929</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -42899,10 +42917,10 @@
         <v>4073</v>
       </c>
       <c r="B75" t="s">
+        <v>3976</v>
+      </c>
+      <c r="C75" t="s">
         <v>4074</v>
-      </c>
-      <c r="C75" t="s">
-        <v>3929</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -42946,7 +42964,7 @@
         <v>4082</v>
       </c>
       <c r="C79" t="s">
-        <v>3934</v>
+        <v>3929</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -42957,7 +42975,7 @@
         <v>4084</v>
       </c>
       <c r="C80" t="s">
-        <v>3929</v>
+        <v>3934</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -43053,7 +43071,7 @@
         <v>4101</v>
       </c>
       <c r="B89" t="s">
-        <v>3968</v>
+        <v>4102</v>
       </c>
       <c r="C89" t="s">
         <v>3929</v>
@@ -43061,10 +43079,10 @@
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>4102</v>
+        <v>4103</v>
       </c>
       <c r="B90" t="s">
-        <v>4103</v>
+        <v>3968</v>
       </c>
       <c r="C90" t="s">
         <v>3929</v>
@@ -43122,6 +43140,39 @@
         <v>4113</v>
       </c>
       <c r="C95" t="s">
+        <v>3929</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" t="s">
+        <v>4114</v>
+      </c>
+      <c r="B96" t="s">
+        <v>4115</v>
+      </c>
+      <c r="C96" t="s">
+        <v>3929</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" t="s">
+        <v>4116</v>
+      </c>
+      <c r="B97" t="s">
+        <v>4117</v>
+      </c>
+      <c r="C97" t="s">
+        <v>3929</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" t="s">
+        <v>4118</v>
+      </c>
+      <c r="B98" t="s">
+        <v>4119</v>
+      </c>
+      <c r="C98" t="s">
         <v>3929</v>
       </c>
     </row>

</xml_diff>